<commit_message>
1. #7604 - zone quantity 2. report translation in malay.
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/WEB-INF/templates/sc/loa/jadual-harga.xlsx
+++ b/portlets/NGeP-portlet/docroot/WEB-INF/templates/sc/loa/jadual-harga.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="60" windowWidth="20112" windowHeight="8016"/>
   </bookViews>
   <sheets>
     <sheet name="ProductSheet" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
   <si>
     <t>Item</t>
   </si>
@@ -23,34 +23,31 @@
     <t>UOM</t>
   </si>
   <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Zone</t>
-  </si>
-  <si>
-    <t>Sub Sequence</t>
-  </si>
-  <si>
-    <t>Unit Price (RM)</t>
-  </si>
-  <si>
-    <t>Total Amount (RM)</t>
-  </si>
-  <si>
-    <t>Frequency per UOM</t>
-  </si>
-  <si>
-    <t>No. UOM per day</t>
-  </si>
-  <si>
-    <t>No. UOM per month</t>
-  </si>
-  <si>
-    <t>No. UOM per year</t>
-  </si>
-  <si>
-    <t>Total Amount (No. of Years )(RM)</t>
+    <t>Kekerapan / Unit Ukuran</t>
+  </si>
+  <si>
+    <t>Bil. Unit Ukuran Sehari</t>
+  </si>
+  <si>
+    <t>Bil. Unit Ukuran Sebulan</t>
+  </si>
+  <si>
+    <t>Zon</t>
+  </si>
+  <si>
+    <t>Kuantiti</t>
+  </si>
+  <si>
+    <t>Tawaran Harga Seunit (RM)</t>
+  </si>
+  <si>
+    <t>Bil. Unit Ukuran Setahun</t>
+  </si>
+  <si>
+    <t>Jumlah Harga Tawaran (RM)</t>
+  </si>
+  <si>
+    <t>Yang Berikutnya</t>
   </si>
 </sst>
 </file>
@@ -410,20 +407,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -432,16 +429,16 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -453,23 +450,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" customWidth="1"/>
     <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -478,25 +475,25 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>